<commit_message>
Modernisering datums, alle jaartallen met 15 verhoogd. Naam database gewijzigd in snoep2025.accdb Diverse afbeeldingen opnieuw gemaakt Normalisatie moet nog bijgeschaafd worden
</commit_message>
<xml_diff>
--- a/data/Werknemers.xlsx
+++ b/data/Werknemers.xlsx
@@ -1,18 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18431"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCEEAF74-2F2C-49C2-9079-23769562F492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12210" xr2:uid="{2A25CBEB-3CC1-4052-813D-F7296D8782A4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{2A25CBEB-3CC1-4052-813D-F7296D8782A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -258,11 +270,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -281,9 +294,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Thema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -321,7 +334,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -427,7 +440,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -569,7 +582,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -578,20 +591,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAE3AC65-A0ED-4370-9473-1EFF982585D1}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,372 +630,375 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="3">
-        <v>25919</v>
+        <v>31398</v>
       </c>
       <c r="H2" s="3">
-        <v>33023</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+        <v>38502</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G3" s="3">
-        <v>26362</v>
+        <v>31840</v>
       </c>
       <c r="H3" s="3">
-        <v>33031</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+        <v>38510</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G4" s="3">
-        <v>26790</v>
+        <v>32269</v>
       </c>
       <c r="H4" s="3">
-        <v>36197</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>41676</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G5" s="3">
-        <v>26119</v>
+        <v>31598</v>
       </c>
       <c r="H5" s="3">
-        <v>32388</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+        <v>37866</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G6" s="3">
-        <v>30653</v>
+        <v>36132</v>
       </c>
       <c r="H6" s="3">
-        <v>37112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+        <v>42591</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>33</v>
       </c>
       <c r="G7" s="3">
-        <v>29040</v>
+        <v>34519</v>
       </c>
       <c r="H7" s="3">
-        <v>34920</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+        <v>40399</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G8" s="3">
-        <v>25325</v>
+        <v>30804</v>
       </c>
       <c r="H8" s="3">
-        <v>31991</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+        <v>37470</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G9" s="3">
-        <v>26945</v>
+        <v>32424</v>
       </c>
       <c r="H9" s="3">
-        <v>35812</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+        <v>41291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>12</v>
       </c>
       <c r="G10" s="3">
-        <v>25476</v>
+        <v>30955</v>
       </c>
       <c r="H10" s="3">
-        <v>31732</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>37211</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="4" t="s">
         <v>33</v>
       </c>
       <c r="G11" s="3">
-        <v>26061</v>
+        <v>31540</v>
       </c>
       <c r="H11" s="3">
-        <v>33000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+        <v>38479</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G12" s="3">
-        <v>24724</v>
+        <v>30203</v>
       </c>
       <c r="H12" s="3">
-        <v>31989</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>37468</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>13</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="4" t="s">
         <v>33</v>
       </c>
       <c r="G13" s="3">
-        <v>26164</v>
+        <v>31643</v>
       </c>
       <c r="H13" s="3">
-        <v>33023</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>38502</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>14</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G14" s="3">
-        <v>27560</v>
+        <v>33039</v>
       </c>
       <c r="H14" s="3">
-        <v>34893</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>40372</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>15</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="4" t="s">
         <v>24</v>
       </c>
       <c r="G15" s="3">
-        <v>30759</v>
+        <v>36237</v>
       </c>
       <c r="H15" s="3">
-        <v>37816</v>
+        <v>43295</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="E2:E15" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>